<commit_message>
Parcours en 7 etapes
</commit_message>
<xml_diff>
--- a/data/banque-exercices.xlsx
+++ b/data/banque-exercices.xlsx
@@ -8,8 +8,9 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Banque" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Générateurs" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mode d'emploi" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Parcours" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Générateurs" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mode d'emploi" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1819,6 +1820,56 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:B3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="26" customWidth="1" min="1" max="1"/>
+    <col width="52" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>Notion</t>
+        </is>
+      </c>
+      <c r="B1" s="4" t="inlineStr">
+        <is>
+          <t>Seuil Explorer (bonnes réponses pour ouvrir Comprendre)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>entiers-naturels</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>ecriture-scientifique</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>6</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:E13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -2185,13 +2236,13 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A7"/>
+  <dimension ref="A1:A8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="120" customWidth="1" min="1" max="1"/>
@@ -2246,6 +2297,13 @@
         </is>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Feuille Parcours : pour chaque notion, le nombre de bonnes réponses dans Explorer qui ouvre l'étape Comprendre.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Notion 6e « Tables de multiplication » et générateurs génériques pour l'Excel
- Nouvelle notion 6e : parcours complet en 7 étapes, 2 exercices (« {} est dans la table de {t} », « {a} × {b} = {} »)
- Énoncés à plusieurs valeurs tirées ({t}, {a}, {b}…)
- Générateurs génériques utilisables depuis l'Excel : liste, entier (pair, impair, multiple de m), decimal, fraction
- Correctifs : définition non dupliquée dans Comprendre, choix de justification plus juste

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01E92HNC9FUW2VcTzfmpL2ox
</commit_message>
<xml_diff>
--- a/data/banque-exercices.xlsx
+++ b/data/banque-exercices.xlsx
@@ -20,7 +20,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -31,6 +31,9 @@
     <font>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="4">
@@ -63,7 +66,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -75,6 +78,7 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -440,7 +444,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T16"/>
+  <dimension ref="A1:T25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -1809,6 +1813,744 @@
         </is>
       </c>
     </row>
+    <row r="17">
+      <c r="A17" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>{} est dans la table de {t}</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>Résultat de la table (t × k, k de 2 à 9)</t>
+        </is>
+      </c>
+      <c r="D17" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="E17" s="3" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
+      <c r="F17" s="3" t="inlineStr">
+        <is>
+          <t>{} = {t} × {k}.</t>
+        </is>
+      </c>
+      <c r="G17" s="3" t="inlineStr">
+        <is>
+          <t>{} est un nombre pair.</t>
+        </is>
+      </c>
+      <c r="H17" s="3" t="inlineStr">
+        <is>
+          <t>{} est plus grand que {t}.</t>
+        </is>
+      </c>
+      <c r="I17" s="3" t="inlineStr">
+        <is>
+          <t>Le dernier chiffre de {} est {t}.</t>
+        </is>
+      </c>
+      <c r="J17" s="3" t="inlineStr">
+        <is>
+          <t>Pourquoi 1</t>
+        </is>
+      </c>
+      <c r="K17" s="3" t="inlineStr"/>
+      <c r="L17" s="3" t="inlineStr"/>
+      <c r="M17" s="3" t="inlineStr"/>
+      <c r="N17" s="3" t="inlineStr"/>
+      <c r="O17" s="3" t="inlineStr">
+        <is>
+          <t>Nombres et calculs</t>
+        </is>
+      </c>
+      <c r="P17" s="3" t="inlineStr">
+        <is>
+          <t>Calcul mental : les tables</t>
+        </is>
+      </c>
+      <c r="Q17" s="3" t="inlineStr">
+        <is>
+          <t>6e</t>
+        </is>
+      </c>
+      <c r="R17" s="3" t="inlineStr">
+        <is>
+          <t>{} est dans la table de {t}, car {t} × {k} = {}. On peut aussi l'écrire {k} × {t}.</t>
+        </is>
+      </c>
+      <c r="S17" s="3" t="inlineStr">
+        <is>
+          <t>tables-multiplication</t>
+        </is>
+      </c>
+      <c r="T17" s="3" t="inlineStr">
+        <is>
+          <t>tm_produit()</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t>{} est dans la table de {t}</t>
+        </is>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D18" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E18" s="3" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
+      <c r="F18" s="3" t="inlineStr">
+        <is>
+          <t>{t} × 0 = 0 : zéro est dans toutes les tables.</t>
+        </is>
+      </c>
+      <c r="G18" s="3" t="inlineStr">
+        <is>
+          <t>0 n'est dans aucune table.</t>
+        </is>
+      </c>
+      <c r="H18" s="3" t="inlineStr">
+        <is>
+          <t>0 est un chiffre.</t>
+        </is>
+      </c>
+      <c r="I18" s="3" t="inlineStr">
+        <is>
+          <t>0 est plus petit que {t}.</t>
+        </is>
+      </c>
+      <c r="J18" s="3" t="inlineStr">
+        <is>
+          <t>Pourquoi 1</t>
+        </is>
+      </c>
+      <c r="K18" s="3" t="inlineStr"/>
+      <c r="L18" s="3" t="inlineStr"/>
+      <c r="M18" s="3" t="inlineStr"/>
+      <c r="N18" s="3" t="inlineStr"/>
+      <c r="O18" s="3" t="inlineStr">
+        <is>
+          <t>Nombres et calculs</t>
+        </is>
+      </c>
+      <c r="P18" s="3" t="inlineStr">
+        <is>
+          <t>Calcul mental : les tables</t>
+        </is>
+      </c>
+      <c r="Q18" s="3" t="inlineStr">
+        <is>
+          <t>6e</t>
+        </is>
+      </c>
+      <c r="R18" s="3" t="inlineStr">
+        <is>
+          <t>{t} × 0 = 0 : zéro est dans toutes les tables, y compris celle de {t}.</t>
+        </is>
+      </c>
+      <c r="S18" s="3" t="inlineStr">
+        <is>
+          <t>tables-multiplication</t>
+        </is>
+      </c>
+      <c r="T18" s="3" t="inlineStr">
+        <is>
+          <t>tm_zero()</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>{} est dans la table de {t}</t>
+        </is>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>Le nombre de la table lui-même</t>
+        </is>
+      </c>
+      <c r="D19" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E19" s="3" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
+      <c r="F19" s="3" t="inlineStr">
+        <is>
+          <t>{} = {t} × 1.</t>
+        </is>
+      </c>
+      <c r="G19" s="3" t="inlineStr">
+        <is>
+          <t>Un nombre n'est jamais dans sa propre table.</t>
+        </is>
+      </c>
+      <c r="H19" s="3" t="inlineStr">
+        <is>
+          <t>{} est un chiffre.</t>
+        </is>
+      </c>
+      <c r="I19" s="3" t="inlineStr">
+        <is>
+          <t>{} est plus petit que 10.</t>
+        </is>
+      </c>
+      <c r="J19" s="3" t="inlineStr">
+        <is>
+          <t>Pourquoi 1</t>
+        </is>
+      </c>
+      <c r="K19" s="3" t="inlineStr"/>
+      <c r="L19" s="3" t="inlineStr"/>
+      <c r="M19" s="3" t="inlineStr"/>
+      <c r="N19" s="3" t="inlineStr"/>
+      <c r="O19" s="3" t="inlineStr">
+        <is>
+          <t>Nombres et calculs</t>
+        </is>
+      </c>
+      <c r="P19" s="3" t="inlineStr">
+        <is>
+          <t>Calcul mental : les tables</t>
+        </is>
+      </c>
+      <c r="Q19" s="3" t="inlineStr">
+        <is>
+          <t>6e</t>
+        </is>
+      </c>
+      <c r="R19" s="3" t="inlineStr">
+        <is>
+          <t>{t} × 1 = {t} : un nombre est toujours dans sa propre table.</t>
+        </is>
+      </c>
+      <c r="S19" s="3" t="inlineStr">
+        <is>
+          <t>tables-multiplication</t>
+        </is>
+      </c>
+      <c r="T19" s="3" t="inlineStr">
+        <is>
+          <t>tm_lui_meme()</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>{} est dans la table de {t}</t>
+        </is>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>Voisin d’un résultat (t × k ± 1)</t>
+        </is>
+      </c>
+      <c r="D20" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="E20" s="3" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="F20" s="3" t="inlineStr">
+        <is>
+          <t>{} est entre {t} × {k1} = {a} et {t} × {k2} = {b} : ce n'est pas un résultat de la table.</t>
+        </is>
+      </c>
+      <c r="G20" s="3" t="inlineStr">
+        <is>
+          <t>{} est un nombre impair.</t>
+        </is>
+      </c>
+      <c r="H20" s="3" t="inlineStr">
+        <is>
+          <t>{} est plus grand que {t}.</t>
+        </is>
+      </c>
+      <c r="I20" s="3" t="inlineStr">
+        <is>
+          <t>Le dernier chiffre de {} n'est pas {t}.</t>
+        </is>
+      </c>
+      <c r="J20" s="3" t="inlineStr">
+        <is>
+          <t>Pourquoi 1</t>
+        </is>
+      </c>
+      <c r="K20" s="3" t="inlineStr"/>
+      <c r="L20" s="3" t="inlineStr"/>
+      <c r="M20" s="3" t="inlineStr"/>
+      <c r="N20" s="3" t="inlineStr"/>
+      <c r="O20" s="3" t="inlineStr">
+        <is>
+          <t>Nombres et calculs</t>
+        </is>
+      </c>
+      <c r="P20" s="3" t="inlineStr">
+        <is>
+          <t>Calcul mental : les tables</t>
+        </is>
+      </c>
+      <c r="Q20" s="3" t="inlineStr">
+        <is>
+          <t>6e</t>
+        </is>
+      </c>
+      <c r="R20" s="3" t="inlineStr">
+        <is>
+          <t>La table de {t} passe par {a} puis {b} : {} est entre les deux, il n'est pas dans la table.</t>
+        </is>
+      </c>
+      <c r="S20" s="3" t="inlineStr">
+        <is>
+          <t>tables-multiplication</t>
+        </is>
+      </c>
+      <c r="T20" s="3" t="inlineStr">
+        <is>
+          <t>tm_voisin()</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>{} est dans la table de {t}</t>
+        </is>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>Se termine par t sans être dans la table</t>
+        </is>
+      </c>
+      <c r="D21" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="E21" s="3" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="F21" s="3" t="inlineStr">
+        <is>
+          <t>Se terminer par {t} ne suffit pas : {} est entre {t} × {k1} = {a} et {t} × {k2} = {b}.</t>
+        </is>
+      </c>
+      <c r="G21" s="3" t="inlineStr">
+        <is>
+          <t>{} se termine par {t}, il est donc dans la table de {t}.</t>
+        </is>
+      </c>
+      <c r="H21" s="3" t="inlineStr">
+        <is>
+          <t>{} est trop petit.</t>
+        </is>
+      </c>
+      <c r="I21" s="3" t="inlineStr">
+        <is>
+          <t>{} est un nombre pair.</t>
+        </is>
+      </c>
+      <c r="J21" s="3" t="inlineStr">
+        <is>
+          <t>Pourquoi 1</t>
+        </is>
+      </c>
+      <c r="K21" s="3" t="inlineStr"/>
+      <c r="L21" s="3" t="inlineStr"/>
+      <c r="M21" s="3" t="inlineStr"/>
+      <c r="N21" s="3" t="inlineStr"/>
+      <c r="O21" s="3" t="inlineStr">
+        <is>
+          <t>Nombres et calculs</t>
+        </is>
+      </c>
+      <c r="P21" s="3" t="inlineStr">
+        <is>
+          <t>Calcul mental : les tables</t>
+        </is>
+      </c>
+      <c r="Q21" s="3" t="inlineStr">
+        <is>
+          <t>6e</t>
+        </is>
+      </c>
+      <c r="R21" s="3" t="inlineStr">
+        <is>
+          <t>{} se termine par {t}, mais la table de {t} passe par {a} puis {b}. Le dernier chiffre ne suffit pas.</t>
+        </is>
+      </c>
+      <c r="S21" s="3" t="inlineStr">
+        <is>
+          <t>tables-multiplication</t>
+        </is>
+      </c>
+      <c r="T21" s="3" t="inlineStr">
+        <is>
+          <t>tm_terminaison()</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>{a} × {b} = {}</t>
+        </is>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>Résultat juste</t>
+        </is>
+      </c>
+      <c r="D22" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="E22" s="3" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
+      <c r="F22" s="3" t="inlineStr">
+        <is>
+          <t>{a} × {b} = {r}.</t>
+        </is>
+      </c>
+      <c r="G22" s="3" t="inlineStr">
+        <is>
+          <t>Le résultat est plus grand que {a} et que {b}.</t>
+        </is>
+      </c>
+      <c r="H22" s="3" t="inlineStr">
+        <is>
+          <t>Le résultat se termine par {b}.</t>
+        </is>
+      </c>
+      <c r="I22" s="3" t="inlineStr">
+        <is>
+          <t>{} est un nombre pair.</t>
+        </is>
+      </c>
+      <c r="J22" s="3" t="inlineStr">
+        <is>
+          <t>Pourquoi 1</t>
+        </is>
+      </c>
+      <c r="K22" s="3" t="inlineStr"/>
+      <c r="L22" s="3" t="inlineStr"/>
+      <c r="M22" s="3" t="inlineStr"/>
+      <c r="N22" s="3" t="inlineStr"/>
+      <c r="O22" s="3" t="inlineStr">
+        <is>
+          <t>Nombres et calculs</t>
+        </is>
+      </c>
+      <c r="P22" s="3" t="inlineStr">
+        <is>
+          <t>Calcul mental : les tables</t>
+        </is>
+      </c>
+      <c r="Q22" s="3" t="inlineStr">
+        <is>
+          <t>6e</t>
+        </is>
+      </c>
+      <c r="R22" s="3" t="inlineStr">
+        <is>
+          <t>{a} × {b} = {r}, et aussi {b} × {a} = {r}.</t>
+        </is>
+      </c>
+      <c r="S22" s="3" t="inlineStr">
+        <is>
+          <t>tables-multiplication</t>
+        </is>
+      </c>
+      <c r="T22" s="3" t="inlineStr">
+        <is>
+          <t>mul_juste()</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B23" s="3" t="inlineStr">
+        <is>
+          <t>{a} × {b} = {}</t>
+        </is>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>Glissement sur la ligne voisine</t>
+        </is>
+      </c>
+      <c r="D23" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="E23" s="3" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="F23" s="3" t="inlineStr">
+        <is>
+          <t>{a} × {b} = {r}. Le nombre {}, c'est {a} × {b2} : on s'est décalé d'une ligne.</t>
+        </is>
+      </c>
+      <c r="G23" s="3" t="inlineStr">
+        <is>
+          <t>Le résultat d'une multiplication est toujours pair.</t>
+        </is>
+      </c>
+      <c r="H23" s="3" t="inlineStr">
+        <is>
+          <t>{} est trop grand.</t>
+        </is>
+      </c>
+      <c r="I23" s="3" t="inlineStr">
+        <is>
+          <t>Il faut inverser les chiffres.</t>
+        </is>
+      </c>
+      <c r="J23" s="3" t="inlineStr">
+        <is>
+          <t>Pourquoi 1</t>
+        </is>
+      </c>
+      <c r="K23" s="3" t="inlineStr"/>
+      <c r="L23" s="3" t="inlineStr"/>
+      <c r="M23" s="3" t="inlineStr"/>
+      <c r="N23" s="3" t="inlineStr"/>
+      <c r="O23" s="3" t="inlineStr">
+        <is>
+          <t>Nombres et calculs</t>
+        </is>
+      </c>
+      <c r="P23" s="3" t="inlineStr">
+        <is>
+          <t>Calcul mental : les tables</t>
+        </is>
+      </c>
+      <c r="Q23" s="3" t="inlineStr">
+        <is>
+          <t>6e</t>
+        </is>
+      </c>
+      <c r="R23" s="3" t="inlineStr">
+        <is>
+          <t>{a} × {b} = {r}. Le nombre {} est le résultat de {a} × {b2} : attention à ne pas glisser sur la ligne voisine.</t>
+        </is>
+      </c>
+      <c r="S23" s="3" t="inlineStr">
+        <is>
+          <t>tables-multiplication</t>
+        </is>
+      </c>
+      <c r="T23" s="3" t="inlineStr">
+        <is>
+          <t>mul_decale()</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B24" s="3" t="inlineStr">
+        <is>
+          <t>{a} × {b} = {}</t>
+        </is>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>Confusion avec l’addition</t>
+        </is>
+      </c>
+      <c r="D24" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E24" s="3" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="F24" s="3" t="inlineStr">
+        <is>
+          <t>{} = {a} + {b} : c'est une addition. {a} × {b} = {r}.</t>
+        </is>
+      </c>
+      <c r="G24" s="3" t="inlineStr">
+        <is>
+          <t>{} est trop petit pour être un résultat de table.</t>
+        </is>
+      </c>
+      <c r="H24" s="3" t="inlineStr">
+        <is>
+          <t>On ne peut pas multiplier {a} par {b}.</t>
+        </is>
+      </c>
+      <c r="I24" s="3" t="inlineStr">
+        <is>
+          <t>{} est un nombre impair.</t>
+        </is>
+      </c>
+      <c r="J24" s="3" t="inlineStr">
+        <is>
+          <t>Pourquoi 1</t>
+        </is>
+      </c>
+      <c r="K24" s="3" t="inlineStr"/>
+      <c r="L24" s="3" t="inlineStr"/>
+      <c r="M24" s="3" t="inlineStr"/>
+      <c r="N24" s="3" t="inlineStr"/>
+      <c r="O24" s="3" t="inlineStr">
+        <is>
+          <t>Nombres et calculs</t>
+        </is>
+      </c>
+      <c r="P24" s="3" t="inlineStr">
+        <is>
+          <t>Calcul mental : les tables</t>
+        </is>
+      </c>
+      <c r="Q24" s="3" t="inlineStr">
+        <is>
+          <t>6e</t>
+        </is>
+      </c>
+      <c r="R24" s="3" t="inlineStr">
+        <is>
+          <t>{} est le résultat de l'addition {a} + {b}. La multiplication donne {a} × {b} = {r}.</t>
+        </is>
+      </c>
+      <c r="S24" s="3" t="inlineStr">
+        <is>
+          <t>tables-multiplication</t>
+        </is>
+      </c>
+      <c r="T24" s="3" t="inlineStr">
+        <is>
+          <t>mul_addition()</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B25" s="3" t="inlineStr">
+        <is>
+          <t>{a} × {b} = {}</t>
+        </is>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>Chiffres inversés</t>
+        </is>
+      </c>
+      <c r="D25" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E25" s="3" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="F25" s="3" t="inlineStr">
+        <is>
+          <t>{a} × {b} = {r} : les chiffres de {} sont inversés.</t>
+        </is>
+      </c>
+      <c r="G25" s="3" t="inlineStr">
+        <is>
+          <t>On ne peut pas multiplier deux chiffres.</t>
+        </is>
+      </c>
+      <c r="H25" s="3" t="inlineStr">
+        <is>
+          <t>{a} est plus petit que {b}.</t>
+        </is>
+      </c>
+      <c r="I25" s="3" t="inlineStr">
+        <is>
+          <t>Il faudrait additionner {a} et {b}.</t>
+        </is>
+      </c>
+      <c r="J25" s="3" t="inlineStr">
+        <is>
+          <t>Pourquoi 1</t>
+        </is>
+      </c>
+      <c r="K25" s="3" t="inlineStr"/>
+      <c r="L25" s="3" t="inlineStr"/>
+      <c r="M25" s="3" t="inlineStr"/>
+      <c r="N25" s="3" t="inlineStr"/>
+      <c r="O25" s="3" t="inlineStr">
+        <is>
+          <t>Nombres et calculs</t>
+        </is>
+      </c>
+      <c r="P25" s="3" t="inlineStr">
+        <is>
+          <t>Calcul mental : les tables</t>
+        </is>
+      </c>
+      <c r="Q25" s="3" t="inlineStr">
+        <is>
+          <t>6e</t>
+        </is>
+      </c>
+      <c r="R25" s="3" t="inlineStr">
+        <is>
+          <t>{a} × {b} = {r}. Ici les chiffres ont été inversés : attention en écrivant le résultat.</t>
+        </is>
+      </c>
+      <c r="S25" s="3" t="inlineStr">
+        <is>
+          <t>tables-multiplication</t>
+        </is>
+      </c>
+      <c r="T25" s="3" t="inlineStr">
+        <is>
+          <t>mul_inverse()</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1820,7 +2562,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B3"/>
+  <dimension ref="A1:B4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -1857,6 +2599,16 @@
       </c>
       <c r="B3" t="n">
         <v>6</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>tables-multiplication</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>8</v>
       </c>
     </row>
   </sheetData>
@@ -1870,10 +2622,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E13"/>
+  <dimension ref="A1:E32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="40" customWidth="1" min="1" max="1"/>
     <col width="22" customWidth="1" min="2" max="2"/>
     <col width="44" customWidth="1" min="3" max="3"/>
     <col width="20" customWidth="1" min="4" max="4"/>
@@ -2228,6 +2980,480 @@
       <c r="E13" t="inlineStr">
         <is>
           <t>{} {b}</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>tm_produit()</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>tables-multiplication</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>t × k, table t de 2 à 9, k de 2 à 9</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>56 (table de 7)</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>{} {t} {k}</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>tm_zero()</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>tables-multiplication</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>0, avec une table t au hasard</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>0 (table de 8)</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>{} {t}</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>tm_lui_meme()</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>tables-multiplication</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Le nombre t lui-même</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>7 (table de 7)</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>{} {t}</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>tm_voisin()</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>tables-multiplication</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>t × k ± 1</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>57 (table de 8)</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>{} {t} {k1} {k2} {a} {b}</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>tm_terminaison()</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>tables-multiplication</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Nombre qui se termine par t sans être dans la table</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>27 (table de 7)</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>{} {t} {k1} {k2} {a} {b}</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>mul_juste()</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>tables-multiplication</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>a × b avec son vrai résultat</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>7 × 8 = 56</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>{} {a} {b} {r}</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>mul_decale()</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>tables-multiplication</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>a × b avec le résultat de a × (b ± 1)</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>7 × 8 = 63</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>{} {a} {b} {b2} {r}</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>mul_addition()</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>tables-multiplication</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>a × b avec le résultat de a + b</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>7 × 8 = 15</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>{} {a} {b} {r}</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>mul_inverse()</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>tables-multiplication</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>a × b avec les chiffres du résultat inversés</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>7 × 8 = 65</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>{} {a} {b} {r}</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t>GÉNÉRATEURS GÉNÉRIQUES (toutes notions)</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr"/>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Sépare les paramètres par « ; » (obligatoire si un nombre a une virgule)</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr"/>
+      <c r="E24" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>liste(12; 18; 2,5; -3; 7/2)</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>toutes</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Un élément de ta liste, au hasard (entiers, décimaux, négatifs, fractions)</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>7/2</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>{}</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>entier(1; 100)</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>toutes</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Entier entre les deux bornes</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>57</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>{} {suivant} {precedent} {double}</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>entier(1; 100; pair)  ·  entier(1; 100; impair)</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>toutes</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Entier pair ou impair</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>42</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>{} {suivant} {precedent} {double}</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>entier(1; 100; multiple de 6)</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>toutes</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Entier qui est un multiple de 6</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>48</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>{} {m} {q} (48 = {m} × {q}) {bas} {haut}</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>entier(1; 100; pas multiple de 6)</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>toutes</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Entier qui n’est pas un multiple de 6</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>40</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>{} {m} {q} {bas} {haut} (40 est entre {bas} et {haut})</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>decimal(0; 10; 2)</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>toutes</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Décimal entre 0 et 10 avec 2 chiffres après la virgule, jamais entier</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>3,47</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>{} {bas} {haut} {arrondi}</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>fraction(1; 40)</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>toutes</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Fraction (dénominateur 2 à 9) qui ne tombe pas juste</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>17/5</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>{} {num} {den} {approx}</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>fraction(1; 40; entière)</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>toutes</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Fraction qui tombe juste</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>24/6</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>{} {num} {den} {valeur}</t>
         </is>
       </c>
     </row>
@@ -2242,7 +3468,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A8"/>
+  <dimension ref="A1:A10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="120" customWidth="1" min="1" max="1"/>
@@ -2304,6 +3530,20 @@
         </is>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>L'énoncé peut contenir d'autres repères que {} : par exemple « {} est dans la table de {t} » ou « {a} × {b} = {} ». Ils sont remplacés par les valeurs tirées (voir l'onglet Générateurs).</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Générateurs génériques (onglet Générateurs) : liste(…), entier(…), decimal(…), fraction(…). Ils permettent de créer un nouvel exercice sans modifier le code de la plateforme.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>